<commit_message>
Girlie Vault: sync keyword-research.xlsx (dynamic funnel counts in Read Me)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/girlievault/keyword-research.xlsx
+++ b/decks/girlievault/keyword-research.xlsx
@@ -21729,9 +21729,9 @@
     <row r="14" ht="65" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>BoFu (48) — category buying guides for shoppers ready to purchase.
-MoFu (54) — best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
-ToFu (18) — education and styling that builds topical authority and earns citations.
+          <t>BoFu (53) — category buying guides for shoppers ready to purchase.
+MoFu (48) — best-of, comparison and use-case articles that capture consideration (and feed AI 'best brand' answers).
+ToFu (19) — education and styling that builds topical authority and earns citations.
 The MoFu/ToFu weighting is deliberate: those terms are winnable at a young domain and are exactly what AI engines cite when shoppers ask for recommendations.</t>
         </is>
       </c>

</xml_diff>